<commit_message>
Export WP8 medication analysis timestamp from updated mapping
Refs #1328
</commit_message>
<xml_diff>
--- a/R-dataprocessor/submodules/manual_start/WP8_export/R-WP8_export/inst/extdata/WP8MRP_Liste_Daten_Mapping20260722.xlsx
+++ b/R-dataprocessor/submodules/manual_start/WP8_export/R-WP8_export/inst/extdata/WP8MRP_Liste_Daten_Mapping20260722.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30613"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{EE6A06D7-04C5-4693-89AC-F1482AA91ECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE2BCB6E-6C63-4317-A6AC-B181C8ECA664}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7AFE0EC7-EE8C-4D48-AC9B-AC9D64DCD770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="65">
   <si>
     <t>Fallvignette</t>
   </si>
@@ -72,6 +72,12 @@
   </si>
   <si>
     <t>Id für den Datensatz, die auf Herkunftsstandort rückschließen lässt</t>
+  </si>
+  <si>
+    <t>wp8_mrp_gruppen_id</t>
+  </si>
+  <si>
+    <t>zufällige ID je Gruppe (für identische MRP einer MA)</t>
   </si>
   <si>
     <t>wp8_mrp_fachbereich</t>
@@ -96,6 +102,18 @@
     </r>
   </si>
   <si>
+    <t>wp8_meda_dat</t>
+  </si>
+  <si>
+    <t>meda_dat</t>
+  </si>
+  <si>
+    <t>timestamp</t>
+  </si>
+  <si>
+    <t>TS der dem MRP zugrundeliegender Medikationsanalyse</t>
+  </si>
+  <si>
     <t>wp8_fv_alter</t>
   </si>
   <si>
@@ -126,14 +144,19 @@
     <t>wp8_fv_diagnosen</t>
   </si>
   <si>
-    <t>Inhalt und Zeiträume mit WP8 
-Besprechen</t>
+    <t>Display einbauen, verhindert NA, wenn im Standort nicht verfügbar</t>
   </si>
   <si>
     <t>wp8_fv_medikation</t>
   </si>
   <si>
+    <t>am Tage der MA</t>
+  </si>
+  <si>
     <t>wp8_fv_laborparameter</t>
+  </si>
+  <si>
+    <t>bis 7 Tage vor MA</t>
   </si>
   <si>
     <t>wp8_fv_op</t>
@@ -280,7 +303,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -596,7 +619,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D98"/>
+  <dimension ref="A1:D100"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="13.15"/>
   <cols>
     <col min="1" max="1" width="54.85546875" customWidth="1"/>
@@ -650,11 +673,14 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" ht="12.75">
       <c r="A5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
         <v>12</v>
       </c>
     </row>
@@ -665,214 +691,237 @@
       <c r="B6" t="s">
         <v>14</v>
       </c>
-      <c r="D6" t="s">
+    </row>
+    <row r="7" spans="1:4" ht="12.75">
+      <c r="A7" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
         <v>16</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>17</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="12.75" customHeight="1">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="12.75">
       <c r="A11" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="3"/>
-    </row>
-    <row r="12" spans="1:4">
+        <v>26</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="12.75" customHeight="1">
       <c r="A12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="3"/>
-    </row>
-    <row r="13" spans="1:4">
+        <v>28</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="12.75">
       <c r="A13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="3"/>
-    </row>
-    <row r="14" spans="1:4">
+        <v>30</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="12.75">
       <c r="A14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
+        <v>32</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="12.75">
       <c r="A15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B15" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
+        <v>34</v>
+      </c>
+      <c r="C15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="3"/>
+    </row>
+    <row r="16" spans="1:4" ht="12.75">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B17" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B19" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B21" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B22" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B23" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="B24" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B27" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B28" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>53</v>
-      </c>
-      <c r="C29">
+        <v>52</v>
+      </c>
+      <c r="B29" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>54</v>
+      </c>
+      <c r="B30" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="4:4" ht="24">
-      <c r="D42" s="2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="43" spans="4:4" ht="12.75"/>
-    <row r="71" spans="2:4">
-      <c r="B71" t="s">
-        <v>55</v>
-      </c>
-      <c r="D71" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="98" spans="3:3">
-      <c r="C98" t="s">
-        <v>53</v>
+    <row r="44" spans="4:4" ht="24">
+      <c r="D44" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="45" spans="4:4" ht="12.75"/>
+    <row r="73" spans="2:4">
+      <c r="B73" t="s">
+        <v>63</v>
+      </c>
+      <c r="D73" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="100" spans="3:3">
+      <c r="C100" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="D10:D13"/>
-  </mergeCells>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <headerFooter>
@@ -883,81 +932,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="93d2b372-37bc-474e-a2f6-e237b07f4f3a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_dlc_DocId xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">TMFEV-885672295-4175</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">
-      <Url>https://tmfev.sharepoint.com/sites/tmf/mi-i/_layouts/15/DocIdRedir.aspx?ID=TMFEV-885672295-4175</Url>
-      <Description>TMFEV-885672295-4175</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Url/>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100370F783D856BE247B308870A0815A245" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="e59e6bd7546e62b090aef4fb5ed9afb6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="15b42a90-06dd-4669-ae82-892e5974bb2f" xmlns:ns3="93d2b372-37bc-474e-a2f6-e237b07f4f3a" xmlns:ns4="2d89f73c-94c0-4155-aa8d-969ee56d6579" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4ca942eca7b8d364d6ad20a4d456e115" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="15b42a90-06dd-4669-ae82-892e5974bb2f"/>
@@ -1222,18 +1196,93 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Url/>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=16.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="93d2b372-37bc-474e-a2f6-e237b07f4f3a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_dlc_DocId xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">TMFEV-885672295-4175</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="15b42a90-06dd-4669-ae82-892e5974bb2f">
+      <Url>https://tmfev.sharepoint.com/sites/tmf/mi-i/_layouts/15/DocIdRedir.aspx?ID=TMFEV-885672295-4175</Url>
+      <Description>TMFEV-885672295-4175</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E64479-D726-4AB8-A716-1F18B611E8E6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAB6B2F1-2C78-4FE6-AF5B-CDBBCB8A75BF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08B8B0EA-3BDF-4954-AE09-AB5AAF359A99}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1817AC26-B6E2-4C47-BB33-95CC1107F6F8}"/>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08B8B0EA-3BDF-4954-AE09-AB5AAF359A99}"/>
-</file>
-
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AAB6B2F1-2C78-4FE6-AF5B-CDBBCB8A75BF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24E64479-D726-4AB8-A716-1F18B611E8E6}"/>
 </file>
</xml_diff>